<commit_message>
docs: finalize V3 architecture docs and update sample data with MNRL outputs
</commit_message>
<xml_diff>
--- a/sample_data/sample_output.xlsx
+++ b/sample_data/sample_output.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ProfitCentre1</t>
+          <t>Unnamed: 3</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -444,14 +444,14 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>IGST Value</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>AvailableCGST</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>CRDRPreGST</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>SGST Amount</t>
@@ -474,7 +474,7 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>ITCReversalIdentifier</t>
+          <t>ITC Eligible</t>
         </is>
       </c>
     </row>

</xml_diff>